<commit_message>
Update README and sample Excel file
Fixed minor formatting in the README changelog section and updated the sample Excel file with new content.
</commit_message>
<xml_diff>
--- a/加分详情参考示例.xlsx
+++ b/加分详情参考示例.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PycharmProjects\Github\Project_scholarship\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8527550A-1BA5-47B6-AED0-4CE84DBA8B85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BD354F0-9F11-44F9-A6C1-C2531FED1E2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,10 +27,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="9">
   <si>
-    <t>项目类别</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>奖项级别</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -60,6 +56,10 @@
   </si>
   <si>
     <t>加分上限</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>项目类型</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -387,27 +387,30 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="4" width="17.5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
       <c r="D1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C2">
         <v>4</v>
@@ -418,10 +421,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C3">
         <v>2</v>
@@ -432,10 +435,10 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C4">
         <v>3</v>
@@ -446,10 +449,10 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C5">
         <v>3</v>
@@ -460,10 +463,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C6">
         <v>2</v>

</xml_diff>